<commit_message>
feat: cap nhat giao dien, wizard dat lich phong van va toi uu cac tinh nang tuyen dung
</commit_message>
<xml_diff>
--- a/src/Ats.Web/wwwroot/templates/Mau_Nhap_Nhan_Su.xlsx
+++ b/src/Ats.Web/wwwroot/templates/Mau_Nhap_Nhan_Su.xlsx
@@ -174,58 +174,58 @@
     <x:t>Senior Software Engineer</x:t>
   </x:si>
   <x:si>
+    <x:t>Candidate</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Ứng viên</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Người nộp hồ sơ từ bên ngoài, không có tài khoản nội bộ (Nộp CV, theo dõi trạng thái hồ sơ, xác nhận lịch phỏng vấn và phản hồi offer)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Nhân viên tuyển dụng</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Người vận hành tuyển dụng hằng ngày (Sàng lọc CV, điều phối pipeline, đặt lịch phỏng vấn, soạn offer)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Trưởng bộ phận</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Người cần người, sở hữu vị trí tuyển dụng (Tạo yêu cầu tuyển dụng, xem ứng viên của vị trí mình, quyết định tuyển)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Người phỏng vấn</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Nhân sự được mời tham gia một vòng phỏng vấn (Xem lịch, đọc CV, nộp phiếu đánh giá theo khung năng lực)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HRManager</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Trưởng phòng Nhân sự</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Chủ sở hữu toàn bộ hoạt động tuyển dụng (Giám sát tất cả vị trí, phân công recruiter, theo dõi ngân sách headcount và báo cáo)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Approver</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Người duyệt</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Ban giám đốc hoặc cấp duyệt theo hạn mức (Phê duyệt yêu cầu tuyển dụng và offer vượt hạn mức lương)</x:t>
+  </x:si>
+  <x:si>
     <x:t>Admin</x:t>
   </x:si>
   <x:si>
-    <x:t>Quản trị viên</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Toàn quyền quản trị hệ thống</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HRManager</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Quản lý nhân sự</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Quản lý tuyển dụng, duyệt yêu cầu và offer</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Quản lý tuyển dụng</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Tạo yêu cầu tuyển dụng, tham gia phỏng vấn</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Người phỏng vấn</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Tham gia phỏng vấn và đánh giá ứng viên</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Chuyên viên tuyển dụng</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Đăng tin, lọc hồ sơ, xếp lịch phỏng vấn</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Approver</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Người phê duyệt</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Phê duyệt yêu cầu tuyển dụng và offer</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Candidate</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Ứng viên</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Ứng viên nội bộ hoặc portal</x:t>
+    <x:t>Quản trị hệ thống</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Người vận hành ứng dụng (Quản lý tài khoản, vai trò, danh mục dùng chung, xem nhật ký hệ thống)</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1193,8 +1193,8 @@
     <x:col min="1" max="1" width="26.282054" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="23.424911" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="16.282054" style="0" customWidth="1"/>
-    <x:col min="4" max="4" width="22.996339" style="0" customWidth="1"/>
-    <x:col min="5" max="5" width="41.424911" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="21.710625" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="122.282054" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:5" ht="26" customHeight="1">
@@ -1239,13 +1239,13 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="C3" s="20" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="D3" s="7" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="D3" s="7" t="s">
+      <x:c r="E3" s="7" t="s">
         <x:v>56</x:v>
-      </x:c>
-      <x:c r="E3" s="7" t="s">
-        <x:v>57</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:5">
@@ -1253,10 +1253,10 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="D4" s="7" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="E4" s="7" t="s">
         <x:v>58</x:v>
-      </x:c>
-      <x:c r="E4" s="7" t="s">
-        <x:v>59</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:5">
@@ -1264,15 +1264,15 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="D5" s="7" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="E5" s="7" t="s">
         <x:v>60</x:v>
-      </x:c>
-      <x:c r="E5" s="7" t="s">
-        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:5">
       <x:c r="C6" s="20" t="s">
-        <x:v>34</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="D6" s="7" t="s">
         <x:v>62</x:v>

</xml_diff>